<commit_message>
Refactor yzy_MambaPro_moe.yml configuration to enhance multi-scale feature extraction and MoE integration, while maintaining baseline parameters. Update documentation for clarity on model advantages and runtime commands.
</commit_message>
<xml_diff>
--- a/试验记录.xlsx
+++ b/试验记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>试验方案</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>通过不同参数 改变moe中三个专家的权重配比</t>
+  </si>
+  <si>
+    <t>jzb调优的参数-baseline</t>
   </si>
 </sst>
 </file>
@@ -90,7 +93,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,13 +103,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
@@ -258,7 +254,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -423,12 +419,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -441,12 +431,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -466,12 +450,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -593,154 +571,160 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -759,6 +743,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1082,198 +1069,364 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="4" max="4" width="18.3888888888889" customWidth="1"/>
     <col min="5" max="5" width="120.111111111111" customWidth="1"/>
-    <col min="8" max="8" width="13.1111111111111" customWidth="1"/>
-    <col min="9" max="9" width="13.6666666666667" customWidth="1"/>
-    <col min="10" max="10" width="12.2222222222222" customWidth="1"/>
-    <col min="11" max="11" width="13.6666666666667" customWidth="1"/>
+    <col min="8" max="8" width="13.1111111111111" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.6666666666667" style="2" customWidth="1"/>
+    <col min="10" max="10" width="12.2222222222222" style="2" customWidth="1"/>
+    <col min="11" max="11" width="13.6666666666667" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="5"/>
+      <c r="H1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" ht="23.4" customHeight="1" spans="1:11">
-      <c r="A4" s="5" t="s">
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+    </row>
+    <row r="4" ht="23.4" customHeight="1" spans="1:15">
+      <c r="A4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5">
+      <c r="G4" s="7"/>
+      <c r="H4" s="7">
         <v>78.9</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="7">
         <v>83.4</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="7">
         <v>89.8</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="7">
         <v>91.9</v>
       </c>
-    </row>
-    <row r="5" ht="24.6" customHeight="1" spans="1:11">
-      <c r="A5" s="6" t="s">
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+    </row>
+    <row r="5" ht="24.6" customHeight="1" spans="1:15">
+      <c r="A5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="7" t="s">
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6">
+      <c r="G5" s="8"/>
+      <c r="H5" s="8">
         <v>80.7</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="8">
         <v>85.2</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="8">
         <v>91.1</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="8">
         <v>94</v>
       </c>
-    </row>
-    <row r="6" ht="25.8" customHeight="1" spans="1:11">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="7" t="s">
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+    </row>
+    <row r="6" ht="25.8" customHeight="1" spans="1:15">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="8">
         <v>80.2</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="8">
         <v>83.9</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="8">
         <v>89.4</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="8">
         <v>92.3</v>
       </c>
-    </row>
-    <row r="7" ht="26.4" customHeight="1" spans="1:7">
-      <c r="A7" s="6" t="s">
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+    </row>
+    <row r="7" ht="26.4" customHeight="1" spans="1:15">
+      <c r="A7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" ht="28.2" customHeight="1" spans="1:7">
-      <c r="A8" s="6" t="s">
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+    </row>
+    <row r="8" ht="28.2" customHeight="1" spans="1:15">
+      <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" ht="27" customHeight="1" spans="1:7">
-      <c r="A9" s="6" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+    </row>
+    <row r="9" ht="27" customHeight="1" spans="1:15">
+      <c r="A9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" ht="50" customHeight="1" spans="1:7">
-      <c r="A10" s="6" t="s">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" ht="50" customHeight="1" spans="1:15">
+      <c r="A10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" ht="28.8" customHeight="1" spans="1:5">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" ht="28.8" customHeight="1" spans="1:15">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="9"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+    </row>
+    <row r="12" ht="36" customHeight="1" spans="1:15">
+      <c r="A12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="1">
+        <v>75.2</v>
+      </c>
+      <c r="I12" s="2">
+        <v>80.1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>88.3</v>
+      </c>
+      <c r="K12" s="2">
+        <v>91.7</v>
+      </c>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+    </row>
+    <row r="13" ht="33" customHeight="1" spans="1:15">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="H13" s="1">
+        <v>74.9</v>
+      </c>
+      <c r="I13" s="2">
+        <v>80.1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>88.3</v>
+      </c>
+      <c r="K13" s="2">
+        <v>90.8</v>
+      </c>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+    </row>
+    <row r="14" ht="27" customHeight="1" spans="1:15">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+    </row>
+    <row r="15" ht="31" customHeight="1" spans="1:15">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+    </row>
+    <row r="16" ht="27" customHeight="1" spans="1:15">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+    </row>
+    <row r="17" ht="28" customHeight="1" spans="1:15">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+    </row>
+    <row r="18" spans="1:15">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="27">
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A5:D5"/>
@@ -1289,11 +1442,16 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="E1:E3"/>
-    <mergeCell ref="H1:H3"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="K1:K3"/>
     <mergeCell ref="A1:D3"/>
     <mergeCell ref="F1:G3"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update configuration documentation for RGBNT201, highlighting similarities and differences among mybest_record01~03.yml files. Remove outdated feature fusion method documentation and example files to streamline project structure.
</commit_message>
<xml_diff>
--- a/试验记录.xlsx
+++ b/试验记录.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27400" windowHeight="9180"/>
+    <workbookView windowWidth="20780" windowHeight="9860"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
   <si>
     <t>试验方案</t>
   </si>
@@ -50,6 +50,15 @@
     <t>Rank-10</t>
   </si>
   <si>
+    <t>4*4</t>
+  </si>
+  <si>
+    <t>8*8</t>
+  </si>
+  <si>
+    <t>16*16</t>
+  </si>
+  <si>
     <t>论文宣称的baseline</t>
   </si>
   <si>
@@ -62,10 +71,12 @@
     <t>滑动窗口(4,8,16) 简单拼接+ moe</t>
   </si>
   <si>
-    <t>./run_experiment.sh   --config_file configs/RGBNT201/MambaPro_moe.yml   --weight_path /home/zubuntu/workspace/yzy/MambaPro/results/everyExperiments/experiment_20251013_110028/models/MambaProbest.pth</t>
-  </si>
-  <si>
-    <t>备注：都是在该 pth 文件下能跑出的结果</t>
+    <t xml:space="preserve">./run_experiment.sh   --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml   </t>
+  </si>
+  <si>
+    <t>训练时：不需要指定最终的 pth，系统会从预训练权重开始训练
+测试时：需要指定要测试的 pth 文件路径
+复现时：可以通过命令行参数覆盖配置文件中的权重路径</t>
   </si>
   <si>
     <t>滑动窗口(4,8)简单拼接 + moe</t>
@@ -83,13 +94,94 @@
     <t>jzb调优的参数-baseline</t>
   </si>
   <si>
-    <t>mybest_record01</t>
-  </si>
-  <si>
-    <t>mybest_record02</t>
-  </si>
-  <si>
-    <t>mybest_record03</t>
+    <t>目标是实现对论文baseline的复现</t>
+  </si>
+  <si>
+    <t>4,8,16简单拼接 + moe + mybest_record01</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh   --config_file configs/RGBNT201/mybest_record01.yml   --weight_path /home/zubuntu/workspace/yzy/MambaPro/mybest_model/experiment_20251013_110028/models/MambaProbest.pth</t>
+  </si>
+  <si>
+    <t>三个 mybest_record 文件，包含的参数结构都是一致的</t>
+  </si>
+  <si>
+    <t>4,8,16简单拼接 + moe + mybest_record02</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh   --config_file configs/RGBNT201/mybest_record02.yml   --weight_path /home/zubuntu/workspace/yzy/MambaPro/mybest_model/experiment_20251014_184036/models/MambaProbest.pth</t>
+  </si>
+  <si>
+    <t>4,8,16简单拼接 + moe + mybest_record03</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh   --config_file configs/RGBNT201/mybest_record03.yml   --weight_path /home/zubuntu/workspace/yzy/MambaPro/mybest_model/experiment_20251015_132633/models/MambaProbest.pth</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[4,8]简单拼接 + 2专家moe </t>
+  </si>
+  <si>
+    <t>./run_experiment.sh \
+  --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml \
+  MODEL.CLIP_MULTI_SCALE_SCALES '[4,8]' \
+  MODEL.MOE_SCALES '[4,8]' \
+  MODEL.MOE_EXPERT_HIDDEN_DIM 1536 \
+  MODEL.MOE_EXPERT_LAYERS 3 \
+  MODEL.MOE_GATE_LAYERS 3 \
+  MODEL.MOE_TEMPERATURE 0.5 \
+  SOLVER.MOE_BALANCE_LOSS_WEIGHT 0.01 \
+  SOLVER.MOE_SPARSITY_LOSS_WEIGHT 0.001 \
+  SOLVER.MOE_DIVERSITY_LOSS_WEIGHT 0.01</t>
+  </si>
+  <si>
+    <t>[4,16]简单拼接 + 2专家moe</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh \
+  --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml \
+  MODEL.CLIP_MULTI_SCALE_SCALES '[4,16]' \
+  MODEL.MOE_SCALES '[4,16]' \
+  MODEL.USE_GATE_FUSION False \
+  MODEL.MOE_EXPERT_HIDDEN_DIM 1280 \
+  MODEL.MOE_TEMPERATURE 0.9 \
+  MODEL.MOE_EXPERT_THRESHOLD 0.15 \
+  MODEL.MOE_GATE_DROPOUT 0.15 \
+  MODEL.MOE_EXPERT_DROPOUT 0.15 \
+  SOLVER.MOE_BALANCE_LOSS_WEIGHT 0.002 \
+  SOLVER.MOE_SPARSITY_LOSS_WEIGHT 0.0002 \
+  SOLVER.MOE_DIVERSITY_LOSS_WEIGHT 0.002</t>
+  </si>
+  <si>
+    <t>[8,16]简单拼接 + 2专家moe</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh \
+  --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml \
+  MODEL.CLIP_MULTI_SCALE_SCALES '[8,16]' \
+  MODEL.MOE_SCALES '[8,16]' \
+  MODEL.USE_GATE_FUSION False \
+  MODEL.MOE_EXPERT_HIDDEN_DIM 1280 \
+  MODEL.MOE_EXPERT_LAYERS 3 \
+  MODEL.MOE_GATE_LAYERS 2 \
+  MODEL.MOE_TEMPERATURE 0.9 \
+  MODEL.MOE_EXPERT_THRESHOLD 0.12 \
+  MODEL.MOE_GATE_DROPOUT 0.12 \
+  MODEL.MOE_EXPERT_DROPOUT 0.12 \
+  SOLVER.MOE_BALANCE_LOSS_WEIGHT 0.003 \
+  SOLVER.MOE_SPARSITY_LOSS_WEIGHT 0.0003 \
+  SOLVER.MOE_DIVERSITY_LOSS_WEIGHT 0.003</t>
+  </si>
+  <si>
+    <t>[4,8,16]门控拼接 + 3专家moe</t>
+  </si>
+  <si>
+    <t>./run_experiment.sh --config_file configs/RGBNT201/yzy_best_Mambapro_moe.yml \
+  MODEL.USE_GATE_FUSION True \
+  MODEL.GATE_NUM_HEADS 4 \
+  MODEL.GATE_DROPOUT 0.05</t>
   </si>
 </sst>
 </file>
@@ -102,7 +194,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +211,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -263,7 +362,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,6 +396,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -595,55 +700,52 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -658,80 +760,86 @@
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -745,6 +853,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1069,354 +1195,569 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:XFD28"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="18.3897058823529" customWidth="1"/>
-    <col min="5" max="5" width="120.110294117647" customWidth="1"/>
-    <col min="8" max="8" width="13.1102941176471" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6691176470588" style="1" customWidth="1"/>
-    <col min="10" max="10" width="12.2205882352941" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6691176470588" style="1" customWidth="1"/>
+    <col min="5" max="5" width="162.036764705882" customWidth="1"/>
+    <col min="8" max="8" width="13.1102941176471" style="2" customWidth="1"/>
+    <col min="9" max="9" width="13.6691176470588" style="2" customWidth="1"/>
+    <col min="10" max="10" width="12.2205882352941" style="2" customWidth="1"/>
+    <col min="11" max="11" width="13.6691176470588" style="2" customWidth="1"/>
+    <col min="12" max="12" width="13.5661764705882" customWidth="1"/>
+    <col min="13" max="13" width="14.1323529411765" customWidth="1"/>
+    <col min="14" max="14" width="14.3235294117647" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="4" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6" t="s">
+      <c r="G1" s="6"/>
+      <c r="H1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
+      <c r="L1" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="O1" s="8"/>
     </row>
     <row r="2" spans="1:15">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="8"/>
     </row>
     <row r="3" spans="1:15">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" ht="23.4" customHeight="1" spans="1:15">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4">
         <v>78.9</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="4">
         <v>83.4</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="4">
         <v>89.8</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="4">
         <v>91.9</v>
       </c>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
     </row>
     <row r="5" ht="24.6" customHeight="1" spans="1:15">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1">
+      <c r="A5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="9">
         <v>80.7</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="9">
         <v>85.2</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="9">
         <v>91.1</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="9">
         <v>94</v>
       </c>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-    </row>
-    <row r="6" ht="25.8" customHeight="1" spans="1:15">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="7" t="s">
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+    </row>
+    <row r="6" ht="52" customHeight="1" spans="1:15">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="9">
+        <v>80.2</v>
+      </c>
+      <c r="I6" s="9">
+        <v>83.9</v>
+      </c>
+      <c r="J6" s="9">
+        <v>89.4</v>
+      </c>
+      <c r="K6" s="9">
+        <v>92.3</v>
+      </c>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" ht="26.4" customHeight="1" spans="1:15">
+      <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+    </row>
+    <row r="8" ht="28.2" customHeight="1" spans="1:15">
+      <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" ht="27" customHeight="1" spans="1:15">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+    </row>
+    <row r="10" ht="50" customHeight="1" spans="1:15">
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+    </row>
+    <row r="11" ht="28.8" customHeight="1" spans="1:15">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+    </row>
+    <row r="12" ht="36" customHeight="1" spans="1:15">
+      <c r="A12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="F12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="1">
-        <v>80.2</v>
-      </c>
-      <c r="I6" s="1">
-        <v>83.9</v>
-      </c>
-      <c r="J6" s="1">
-        <v>89.4</v>
-      </c>
-      <c r="K6" s="1">
-        <v>92.3</v>
-      </c>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-    </row>
-    <row r="7" ht="26.4" customHeight="1" spans="1:15">
-      <c r="A7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-    </row>
-    <row r="8" ht="28.2" customHeight="1" spans="1:15">
-      <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-    </row>
-    <row r="9" ht="27" customHeight="1" spans="1:15">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-    </row>
-    <row r="10" ht="50" customHeight="1" spans="1:15">
-      <c r="A10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-    </row>
-    <row r="11" ht="28.8" customHeight="1" spans="1:15">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-    </row>
-    <row r="12" ht="36" customHeight="1" spans="1:15">
-      <c r="A12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="F12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1">
+      <c r="G12" s="2"/>
+      <c r="H12" s="2">
         <v>75.2</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="2">
         <v>80.1</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>88.3</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>91.7</v>
       </c>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
     </row>
     <row r="13" ht="33" customHeight="1" spans="1:15">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="H13" s="1">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="2">
         <v>74.9</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="2">
         <v>80.1</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>88.3</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>90.8</v>
       </c>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
     </row>
     <row r="14" ht="31" customHeight="1" spans="1:15">
-      <c r="A14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
+      <c r="A14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
     </row>
     <row r="15" ht="31" customHeight="1" spans="1:15">
-      <c r="A15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-    </row>
-    <row r="16" ht="27" customHeight="1" spans="1:15">
-      <c r="A16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-    </row>
-    <row r="17" ht="28" customHeight="1" spans="1:15">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-    </row>
-    <row r="18" spans="1:15">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+    </row>
+    <row r="16" ht="31" customHeight="1" spans="1:15">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+    </row>
+    <row r="17" ht="31" customHeight="1" spans="1:15">
+      <c r="A17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+    </row>
+    <row r="18" ht="27" customHeight="1" spans="1:15">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+    </row>
+    <row r="19" ht="27" customHeight="1" spans="1:15">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+    </row>
+    <row r="20" ht="27" customHeight="1" spans="1:15">
+      <c r="A20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="2">
+        <v>76.5</v>
+      </c>
+      <c r="I20" s="2">
+        <v>78.2</v>
+      </c>
+      <c r="J20" s="2">
+        <v>85.3</v>
+      </c>
+      <c r="K20" s="2">
+        <v>90.8</v>
+      </c>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+    </row>
+    <row r="21" ht="28" customHeight="1" spans="1:15">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+    </row>
+    <row r="22" ht="27" customHeight="1" spans="1:15">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="2">
+        <v>78.3</v>
+      </c>
+      <c r="I22" s="2">
+        <v>81.3</v>
+      </c>
+      <c r="J22" s="2">
+        <v>89.2</v>
+      </c>
+      <c r="K22" s="2">
+        <v>92.6</v>
+      </c>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+    </row>
+    <row r="23" ht="33" customHeight="1" spans="1:11">
+      <c r="A23" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" s="2">
+        <v>73.1</v>
+      </c>
+      <c r="I23" s="2">
+        <v>75.1</v>
+      </c>
+      <c r="J23" s="2">
+        <v>83.4</v>
+      </c>
+      <c r="K23" s="2">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1" spans="1:11">
+      <c r="A24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="H24" s="2">
+        <v>73.6</v>
+      </c>
+      <c r="I24" s="2">
+        <v>76.1</v>
+      </c>
+      <c r="J24" s="2">
+        <v>84</v>
+      </c>
+      <c r="K24" s="2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1" spans="1:14">
+      <c r="A25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" s="2">
+        <v>75.6</v>
+      </c>
+      <c r="I25" s="2">
+        <v>78.6</v>
+      </c>
+      <c r="J25" s="2">
+        <v>87.6</v>
+      </c>
+      <c r="K25" s="2">
+        <v>92</v>
+      </c>
+      <c r="M25" s="1">
+        <v>0.144</v>
+      </c>
+      <c r="N25" s="1">
+        <v>0.855</v>
+      </c>
+    </row>
+    <row r="26" ht="29" customHeight="1" spans="1:14">
+      <c r="A26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="L26" s="14">
+        <v>0.488</v>
+      </c>
+      <c r="M26" s="14">
+        <v>0.205</v>
+      </c>
+      <c r="N26" s="14">
+        <v>0.306</v>
+      </c>
+    </row>
+    <row r="27" s="1" customFormat="1" ht="32" customHeight="1"/>
+    <row r="28" ht="29" customHeight="1" spans="1:4">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="54">
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A5:D5"/>
@@ -1432,16 +1773,43 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="A11:D11"/>
+    <mergeCell ref="F11:G11"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="A13:D13"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="A14:D14"/>
+    <mergeCell ref="F14:G14"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="A16:D16"/>
+    <mergeCell ref="F16:G16"/>
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="F18:G18"/>
     <mergeCell ref="A19:D19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A27:XFD27"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="E1:E3"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="L1:L3"/>
+    <mergeCell ref="M1:M3"/>
+    <mergeCell ref="N1:N3"/>
     <mergeCell ref="A1:D3"/>
     <mergeCell ref="F1:G3"/>
   </mergeCells>

</xml_diff>

<commit_message>
Refactor font setup in visualization scripts to simplify Chinese font handling, directly set font parameters, and suppress related warnings for improved clarity and rendering consistency.
</commit_message>
<xml_diff>
--- a/试验记录.xlsx
+++ b/试验记录.xlsx
@@ -1195,7 +1195,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XFD28"/>
+  <dimension ref="A1:XFD29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="4" max="4" width="18.3897058823529" customWidth="1"/>
@@ -1649,112 +1649,149 @@
       <c r="K22" s="2">
         <v>92.6</v>
       </c>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
+      <c r="L22" s="8">
+        <v>0.04</v>
+      </c>
+      <c r="M22" s="8">
+        <v>0.04</v>
+      </c>
+      <c r="N22" s="8">
+        <v>0.9</v>
+      </c>
       <c r="O22" s="8"/>
     </row>
     <row r="23" ht="33" customHeight="1" spans="1:11">
-      <c r="A23" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="11"/>
+      <c r="H23" s="2">
+        <v>77.6</v>
+      </c>
+      <c r="I23" s="2">
+        <v>81.6</v>
+      </c>
+      <c r="J23" s="2">
+        <v>89.1</v>
+      </c>
+      <c r="K23" s="2">
+        <v>92.5</v>
+      </c>
+    </row>
+    <row r="24" ht="33" customHeight="1" spans="1:11">
+      <c r="A24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H24" s="2">
         <v>73.1</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I24" s="2">
         <v>75.1</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J24" s="2">
         <v>83.4</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K24" s="2">
         <v>88.5</v>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1" spans="1:11">
-      <c r="A24" s="1" t="s">
+    <row r="25" ht="28" customHeight="1" spans="1:11">
+      <c r="A25" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="H24" s="2">
-        <v>73.6</v>
-      </c>
-      <c r="I24" s="2">
-        <v>76.1</v>
-      </c>
-      <c r="J24" s="2">
-        <v>84</v>
-      </c>
-      <c r="K24" s="2">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1" spans="1:14">
-      <c r="A25" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H25" s="2">
-        <v>75.6</v>
+        <v>73.6</v>
       </c>
       <c r="I25" s="2">
-        <v>78.6</v>
+        <v>76.1</v>
       </c>
       <c r="J25" s="2">
-        <v>87.6</v>
+        <v>84</v>
       </c>
       <c r="K25" s="2">
-        <v>92</v>
-      </c>
-      <c r="M25" s="1">
-        <v>0.144</v>
-      </c>
-      <c r="N25" s="1">
-        <v>0.855</v>
-      </c>
-    </row>
-    <row r="26" ht="29" customHeight="1" spans="1:14">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1" spans="1:14">
       <c r="A26" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" s="2">
+        <v>75.6</v>
+      </c>
+      <c r="I26" s="2">
+        <v>78.6</v>
+      </c>
+      <c r="J26" s="2">
+        <v>87.6</v>
+      </c>
+      <c r="K26" s="2">
+        <v>92</v>
+      </c>
+      <c r="M26" s="1">
+        <v>0.144</v>
+      </c>
+      <c r="N26" s="1">
+        <v>0.855</v>
+      </c>
+    </row>
+    <row r="27" ht="29" customHeight="1" spans="1:14">
+      <c r="A27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="L26" s="14">
+      <c r="H27" s="2">
+        <v>73.8</v>
+      </c>
+      <c r="I27" s="2">
+        <v>75.7</v>
+      </c>
+      <c r="J27" s="2">
+        <v>84.7</v>
+      </c>
+      <c r="K27" s="2">
+        <v>88.6</v>
+      </c>
+      <c r="L27" s="14">
         <v>0.488</v>
       </c>
-      <c r="M26" s="14">
+      <c r="M27" s="14">
         <v>0.205</v>
       </c>
-      <c r="N26" s="14">
+      <c r="N27" s="14">
         <v>0.306</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="1" ht="32" customHeight="1"/>
-    <row r="28" ht="29" customHeight="1" spans="1:4">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+    <row r="28" s="1" customFormat="1" ht="32" customHeight="1"/>
+    <row r="29" ht="29" customHeight="1" spans="1:4">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -1796,12 +1833,12 @@
     <mergeCell ref="F21:G21"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="F22:G22"/>
-    <mergeCell ref="A23:D23"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A27:XFD27"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A28:XFD28"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="E1:E3"/>
     <mergeCell ref="H1:H3"/>
     <mergeCell ref="I1:I3"/>

</xml_diff>

<commit_message>
Remove MambaPro_moe.yml configuration file and update documentation with new experiment setups and results for RGBNT201 configurations, enhancing clarity on model performance and command execution.
</commit_message>
<xml_diff>
--- a/试验记录.xlsx
+++ b/试验记录.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>试验方案</t>
   </si>
@@ -50,6 +50,15 @@
     <t>Rank-10</t>
   </si>
   <si>
+    <t>4*4 专家</t>
+  </si>
+  <si>
+    <t>8*8专家</t>
+  </si>
+  <si>
+    <t>16*16专家</t>
+  </si>
+  <si>
     <t>论文宣称的baseline</t>
   </si>
   <si>
@@ -81,6 +90,12 @@
   </si>
   <si>
     <t>jzb调优的参数-baseline</t>
+  </si>
+  <si>
+    <t>yzy_moe</t>
+  </si>
+  <si>
+    <t>mybestrecord_01</t>
   </si>
 </sst>
 </file>
@@ -254,7 +269,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -288,6 +303,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -592,7 +613,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -616,16 +637,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -634,85 +655,85 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -723,32 +744,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1075,358 +1096,383 @@
     <col min="4" max="4" width="18.3888888888889" customWidth="1"/>
     <col min="5" max="5" width="120.111111111111" customWidth="1"/>
     <col min="8" max="8" width="13.1111111111111" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6666666666667" style="2" customWidth="1"/>
-    <col min="10" max="10" width="12.2222222222222" style="2" customWidth="1"/>
-    <col min="11" max="11" width="13.6666666666667" style="2" customWidth="1"/>
+    <col min="9" max="9" width="13.6666666666667" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.2222222222222" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6666666666667" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.3148148148148" customWidth="1"/>
+    <col min="13" max="13" width="16.7314814814815" customWidth="1"/>
+    <col min="14" max="14" width="16.8518518518519" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6" t="s">
+      <c r="G1" s="4"/>
+      <c r="H1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
+      <c r="L1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="O1" s="7"/>
     </row>
     <row r="2" spans="1:15">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
       <c r="L2" s="10"/>
       <c r="M2" s="10"/>
       <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
+      <c r="O2" s="7"/>
     </row>
     <row r="3" spans="1:15">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
+      <c r="O3" s="7"/>
     </row>
     <row r="4" ht="23.4" customHeight="1" spans="1:15">
-      <c r="A4" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6">
         <v>78.9</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>83.4</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="6">
         <v>89.8</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="6">
         <v>91.9</v>
       </c>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
     </row>
     <row r="5" ht="24.6" customHeight="1" spans="1:15">
-      <c r="A5" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8">
+      <c r="A5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1">
         <v>80.7</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="1">
         <v>85.2</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="1">
         <v>91.1</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="1">
         <v>94</v>
       </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
     </row>
     <row r="6" ht="25.8" customHeight="1" spans="1:15">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="9" t="s">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="1">
+        <v>80.2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>83.9</v>
+      </c>
+      <c r="J6" s="1">
+        <v>89.4</v>
+      </c>
+      <c r="K6" s="1">
+        <v>92.3</v>
+      </c>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+    </row>
+    <row r="7" ht="26.4" customHeight="1" spans="1:15">
+      <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+    </row>
+    <row r="8" ht="28.2" customHeight="1" spans="1:15">
+      <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+    </row>
+    <row r="9" ht="27" customHeight="1" spans="1:15">
+      <c r="A9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+    </row>
+    <row r="10" ht="50" customHeight="1" spans="1:15">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+    </row>
+    <row r="11" ht="28.8" customHeight="1" spans="1:15">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+    </row>
+    <row r="12" ht="36" customHeight="1" spans="1:15">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="F12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="8">
-        <v>80.2</v>
-      </c>
-      <c r="I6" s="8">
-        <v>83.9</v>
-      </c>
-      <c r="J6" s="8">
-        <v>89.4</v>
-      </c>
-      <c r="K6" s="8">
-        <v>92.3</v>
-      </c>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-    </row>
-    <row r="7" ht="26.4" customHeight="1" spans="1:15">
-      <c r="A7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-    </row>
-    <row r="8" ht="28.2" customHeight="1" spans="1:15">
-      <c r="A8" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-    </row>
-    <row r="9" ht="27" customHeight="1" spans="1:15">
-      <c r="A9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-    </row>
-    <row r="10" ht="50" customHeight="1" spans="1:15">
-      <c r="A10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" ht="28.8" customHeight="1" spans="1:15">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-    </row>
-    <row r="12" ht="36" customHeight="1" spans="1:15">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="F12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="1"/>
       <c r="H12" s="1">
         <v>75.2</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>80.1</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>88.3</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>91.7</v>
       </c>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
     </row>
     <row r="13" ht="33" customHeight="1" spans="1:15">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
       <c r="H13" s="1">
         <v>74.9</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>80.1</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>88.3</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>90.8</v>
       </c>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
     </row>
     <row r="14" ht="27" customHeight="1" spans="1:15">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
+      <c r="A14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="1">
+        <v>70.7</v>
+      </c>
+      <c r="I14" s="1">
+        <v>74.8</v>
+      </c>
+      <c r="J14" s="1">
+        <v>84.3</v>
+      </c>
+      <c r="K14" s="1">
+        <v>88.5</v>
+      </c>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
     </row>
     <row r="15" ht="31" customHeight="1" spans="1:15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
+      <c r="A15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="H15" s="1">
+        <v>73.4</v>
+      </c>
+      <c r="I15" s="1">
+        <v>75.5</v>
+      </c>
+      <c r="J15" s="1">
+        <v>85.3</v>
+      </c>
+      <c r="K15" s="1">
+        <v>88.9</v>
+      </c>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="7"/>
     </row>
     <row r="16" ht="27" customHeight="1" spans="1:15">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
     </row>
     <row r="17" ht="28" customHeight="1" spans="1:15">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
     </row>
     <row r="18" spans="1:15">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="36">
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A5:D5"/>
@@ -1445,13 +1491,22 @@
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="A13:D13"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="A14:D14"/>
+    <mergeCell ref="F14:G14"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="E1:E3"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="L1:L3"/>
+    <mergeCell ref="M1:M3"/>
+    <mergeCell ref="N1:N3"/>
     <mergeCell ref="A1:D3"/>
     <mergeCell ref="F1:G3"/>
   </mergeCells>

</xml_diff>